<commit_message>
style(task 701 insulin): implemented Ina's changes to case document which improved formatting and clarity
</commit_message>
<xml_diff>
--- a/Tasks/Task_701_insulin_synthesis/metabolites_additions.xlsx
+++ b/Tasks/Task_701_insulin_synthesis/metabolites_additions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Git\MSP_p3_2026_hormone_cytokine_task_creation\Tasks\Task_701_insulin_synthesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\MSP_p3_2026_hormone_cytokine_task_creation\Tasks\Task_701_insulin_synthesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF2B31E-45A4-4BA1-BE1B-F4090370FB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC768EF-D9C8-4DB9-9CA3-C81A4A144C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{CD5DF94A-FED4-4ED9-B2C5-1CBFE42F25CF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{CD5DF94A-FED4-4ED9-B2C5-1CBFE42F25CF}"/>
   </bookViews>
   <sheets>
     <sheet name="mets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="92">
   <si>
     <t>action</t>
   </si>
@@ -307,13 +307,19 @@
   </si>
   <si>
     <t>gene-pseudo-metabolite-intermediate</t>
+  </si>
+  <si>
+    <t>des-65-55-pro-insulin[s]</t>
+  </si>
+  <si>
+    <t>des-32-33-pro-insulin[s]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -343,24 +349,9 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="7.7"/>
-      <color rgb="FF666666"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="13.5"/>
       <color rgb="FF161D39"/>
       <name val="Source Sans Pro"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
       <family val="2"/>
     </font>
     <font>
@@ -368,6 +359,25 @@
       <color rgb="FF0A0A0A"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7.7"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -396,7 +406,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -413,16 +423,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -893,20 +908,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D14686DA-B500-41AE-B187-0230B8D69B0A}">
   <dimension ref="A1:O267"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="22.5" customWidth="1"/>
-    <col min="8" max="8" width="28.125" customWidth="1"/>
-    <col min="9" max="9" width="39.125" customWidth="1"/>
-    <col min="10" max="10" width="11.5" style="2"/>
-    <col min="11" max="11" width="14.5" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.5" style="2"/>
-    <col min="13" max="13" width="32.125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="16.25" customWidth="1"/>
-    <col min="18" max="20" width="23.875" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" customWidth="1"/>
+    <col min="8" max="8" width="28.140625" customWidth="1"/>
+    <col min="9" max="9" width="39.140625" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" style="2"/>
+    <col min="11" max="11" width="14.42578125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" style="2"/>
+    <col min="13" max="13" width="32.140625" style="4" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="18" max="20" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -950,268 +965,400 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="36" x14ac:dyDescent="0.25">
       <c r="G2" s="6"/>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="6"/>
-      <c r="K2" s="2" t="s">
+      <c r="I2" s="9"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="L2" s="10"/>
+      <c r="M2" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="12" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="36" x14ac:dyDescent="0.25">
       <c r="G3" s="6"/>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="I3" s="13"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="L3" s="10"/>
+      <c r="M3" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="12" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G4" s="6"/>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="M4" s="4" t="s">
+      <c r="I4" s="9"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
     </row>
     <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G5" s="6"/>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I5" s="6"/>
-      <c r="M5" s="4" t="s">
+      <c r="I5" s="9"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
     </row>
     <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="I6" s="9"/>
-      <c r="M6" s="4" t="s">
+      <c r="I6" s="14"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="9"/>
-      <c r="K7" s="10" t="s">
+      <c r="I7" s="14"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="L7" s="10"/>
+      <c r="M7" s="11" t="s">
         <v>66</v>
       </c>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
     </row>
     <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="I8" s="6"/>
-      <c r="M8" s="4" t="s">
+      <c r="I8" s="9"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="11" t="s">
         <v>85</v>
       </c>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="I9" s="6"/>
-      <c r="M9" s="4" t="s">
+      <c r="I9" s="9"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="11" t="s">
         <v>85</v>
       </c>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
     </row>
     <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H10" s="6" t="s">
+      <c r="H10" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="6"/>
-      <c r="M10" s="4" t="s">
+      <c r="I10" s="9"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="11" t="s">
         <v>85</v>
       </c>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
     </row>
     <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H11" s="6" t="s">
+      <c r="H11" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="I11" s="6"/>
-      <c r="M11" s="4" t="s">
+      <c r="I11" s="9"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="11" t="s">
         <v>85</v>
       </c>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
     </row>
     <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="I12" s="6"/>
-      <c r="M12" s="12" t="s">
+      <c r="I12" s="9"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
     </row>
     <row r="13" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="I13" s="11"/>
-      <c r="M13" s="12" t="s">
+      <c r="I13" s="15"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
     </row>
     <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H14" s="6" t="s">
+      <c r="H14" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="I14" s="6"/>
-      <c r="M14" s="12" t="s">
+      <c r="I14" s="9"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
     </row>
     <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="I15" s="6"/>
-      <c r="M15" s="12" t="s">
+      <c r="I15" s="9"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="11" t="s">
         <v>89</v>
       </c>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
     </row>
     <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H16" s="6" t="s">
+      <c r="H16" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="I16" s="6"/>
-      <c r="M16" s="12" t="s">
+      <c r="I16" s="9"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="11" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="17" spans="8:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H17" s="11" t="s">
+      <c r="N16" s="13"/>
+      <c r="O16" s="13"/>
+    </row>
+    <row r="17" spans="8:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H17" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="I17" s="11"/>
-      <c r="M17" s="12" t="s">
+      <c r="I17" s="15"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="11" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="18" spans="8:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H18" s="11" t="s">
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+    </row>
+    <row r="18" spans="8:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H18" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="11"/>
-      <c r="M18" s="12" t="s">
+      <c r="I18" s="15"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="11" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="19" spans="8:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H19" s="6" t="s">
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+    </row>
+    <row r="19" spans="8:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H19" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="I19" s="13"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
+    </row>
+    <row r="20" spans="8:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H20" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="I20" s="13"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+    </row>
+    <row r="21" spans="8:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H21" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="I19" s="6"/>
-      <c r="K19" s="2" t="s">
+      <c r="I21" s="9"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="L21" s="10"/>
+      <c r="M21" s="11" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="20" spans="8:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H20" s="6" t="s">
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+    </row>
+    <row r="22" spans="8:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H22" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="I20" s="6"/>
-      <c r="K20" s="2" t="s">
+      <c r="I22" s="9"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="L22" s="10"/>
+      <c r="M22" s="11" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="21" spans="8:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H21" s="6"/>
-    </row>
-    <row r="124" spans="13:13" x14ac:dyDescent="0.2">
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+    </row>
+    <row r="23" spans="8:15" x14ac:dyDescent="0.25">
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+    </row>
+    <row r="24" spans="8:15" x14ac:dyDescent="0.25">
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+    </row>
+    <row r="124" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M124"/>
     </row>
-    <row r="125" spans="13:13" x14ac:dyDescent="0.2">
+    <row r="125" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M125"/>
     </row>
-    <row r="145" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="145" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K145"/>
     </row>
-    <row r="146" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="146" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K146"/>
     </row>
-    <row r="147" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="147" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K147"/>
     </row>
-    <row r="148" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="148" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K148"/>
     </row>
-    <row r="149" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="149" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K149"/>
     </row>
-    <row r="150" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="150" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K150"/>
     </row>
-    <row r="151" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="151" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K151"/>
     </row>
-    <row r="152" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="152" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K152"/>
     </row>
-    <row r="258" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="258" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K258"/>
     </row>
-    <row r="259" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="259" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K259"/>
     </row>
-    <row r="260" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="260" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K260"/>
     </row>
-    <row r="261" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="261" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K261"/>
     </row>
-    <row r="262" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="262" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K262"/>
     </row>
-    <row r="263" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="263" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K263"/>
     </row>
-    <row r="264" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="264" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K264"/>
     </row>
-    <row r="265" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="265" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K265"/>
     </row>
-    <row r="266" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="266" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K266"/>
     </row>
-    <row r="267" spans="11:11" x14ac:dyDescent="0.2">
+    <row r="267" spans="11:11" x14ac:dyDescent="0.25">
       <c r="K267"/>
     </row>
   </sheetData>
@@ -1274,13 +1421,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47C4FABE-BBAA-42F0-8C19-3F54C559520F}">
   <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5" customWidth="1"/>
-    <col min="2" max="2" width="26.125" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1288,7 +1435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1297,7 +1444,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -1306,7 +1453,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
@@ -1315,7 +1462,7 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
@@ -1324,7 +1471,7 @@
       </c>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1333,7 +1480,7 @@
       </c>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
@@ -1342,7 +1489,7 @@
       </c>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
@@ -1351,7 +1498,7 @@
       </c>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -1360,7 +1507,7 @@
       </c>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>30</v>
       </c>
@@ -1369,7 +1516,7 @@
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
@@ -1378,7 +1525,7 @@
       </c>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>34</v>
       </c>
@@ -1387,7 +1534,7 @@
       </c>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>36</v>
       </c>
@@ -1396,7 +1543,7 @@
       </c>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>38</v>
       </c>
@@ -1405,7 +1552,7 @@
       </c>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>40</v>
       </c>
@@ -1414,7 +1561,7 @@
       </c>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>42</v>
       </c>
@@ -1423,7 +1570,7 @@
       </c>
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>44</v>
       </c>
@@ -1432,7 +1579,7 @@
       </c>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>46</v>
       </c>
@@ -1441,7 +1588,7 @@
       </c>
       <c r="C18" s="1"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>48</v>
       </c>
@@ -1450,7 +1597,7 @@
       </c>
       <c r="C19" s="1"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>50</v>
       </c>
@@ -1459,7 +1606,7 @@
       </c>
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>52</v>
       </c>
@@ -1468,7 +1615,7 @@
       </c>
       <c r="C21" s="1"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>54</v>
       </c>
@@ -1477,7 +1624,7 @@
       </c>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>56</v>
       </c>
@@ -1486,7 +1633,7 @@
       </c>
       <c r="C23" s="1"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>58</v>
       </c>

</xml_diff>